<commit_message>
Completed with some pending tasks ( before Starting the B2 feature )
B4-T007	Configure Named Credentials — B4 Integrations	Partially complete. DocuSign done; AWS Textract, Azure OCR, Virus Scan, Adobe Sign paused/not configured live.
B4-T043	Adobe Sign Service	Code exists, live Adobe setup paused.
B4-T044	Adobe Sign Webhook Handler	Code exists, live Adobe setup paused.
B4-T058	Upgrade DocuSign Connector to AgentExchange MCP Tool	Deferred; optional add-on requiring AgentExchange connector/package.
</commit_message>
<xml_diff>
--- a/docs/Design_docs/KT_B4_DocumentManagement_Tracker.xlsx
+++ b/docs/Design_docs/KT_B4_DocumentManagement_Tracker.xlsx
@@ -1,26 +1,32 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <workbookPr/>
-  <sheets>
-    <sheet state="hidden" name="📊 Dashboard" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="📋 All Tasks" sheetId="2" r:id="rId5"/>
-    <sheet state="visible" name="📅 Sprint Plan" sheetId="3" r:id="rId6"/>
-    <sheet state="visible" name="🔗 Integration Reference" sheetId="4" r:id="rId7"/>
-  </sheets>
-  <definedNames>
-    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'📋 All Tasks'!$A$1:$U$1</definedName>
-  </definedNames>
-  <calcPr/>
-  <extLst>
-    <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataChecksum="RbS83eN0b/A8QkqvStPlmvUPn668ajBW2hwc0KexJe8="/>
-    </ext>
-  </extLst>
-</workbook>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-05-04T15:55:36Z</dcterms:created>
+  <dc:creator>openpyxl</dc:creator>
+</cp:coreProperties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\custom.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes"/>
+</file>
+
+<file path=xl\drawings\drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl\drawings\drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl\drawings\drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl\drawings\drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1058" uniqueCount="403">
   <si>
     <t>KT Onboarding Enterprise — B4 Document Management &amp; CLM</t>
@@ -1234,7 +1240,7 @@
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <fonts count="15">
     <font>
@@ -1603,23 +1609,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
@@ -1813,7 +1803,28 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <workbookPr/>
+  <sheets>
+    <sheet state="hidden" name="📊 Dashboard" sheetId="1" r:id="rId4"/>
+    <sheet state="visible" name="📋 All Tasks" sheetId="2" r:id="rId5"/>
+    <sheet state="visible" name="📅 Sprint Plan" sheetId="3" r:id="rId6"/>
+    <sheet state="visible" name="🔗 Integration Reference" sheetId="4" r:id="rId7"/>
+  </sheets>
+  <definedNames>
+    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'📋 All Tasks'!$A$1:$U$1</definedName>
+  </definedNames>
+  <calcPr/>
+  <extLst>
+    <ext uri="GoogleSheetsCustomDataVersion2">
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataChecksum="RbS83eN0b/A8QkqvStPlmvUPn668ajBW2hwc0KexJe8="/>
+    </ext>
+  </extLst>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <pageSetUpPr/>
@@ -3409,7 +3420,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <pageSetUpPr/>
@@ -3530,8 +3541,10 @@
       <c r="I2" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J2" s="26" t="s">
-        <v>73</v>
+      <c r="J2" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K2" s="27"/>
       <c r="L2" s="26" t="s">
@@ -3555,11 +3568,13 @@
         <v>5.625</v>
       </c>
       <c r="S2" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T2" s="27"/>
-      <c r="U2" s="27" t="s">
-        <v>74</v>
+      <c r="U2" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -3590,8 +3605,10 @@
       <c r="I3" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J3" s="26" t="s">
-        <v>73</v>
+      <c r="J3" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K3" s="27"/>
       <c r="L3" s="26" t="s">
@@ -3615,11 +3632,13 @@
         <v>5.625</v>
       </c>
       <c r="S3" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T3" s="27"/>
-      <c r="U3" s="27" t="s">
-        <v>78</v>
+      <c r="U3" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -3650,8 +3669,10 @@
       <c r="I4" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J4" s="26" t="s">
-        <v>73</v>
+      <c r="J4" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K4" s="27"/>
       <c r="L4" s="26" t="s">
@@ -3675,12 +3696,16 @@
         <v>5.625</v>
       </c>
       <c r="S4" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T4" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="U4" s="27"/>
+      <c r="U4" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="76.5" customHeight="1">
       <c r="A5" s="26" t="s">
@@ -3710,8 +3735,10 @@
       <c r="I5" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J5" s="26" t="s">
-        <v>73</v>
+      <c r="J5" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K5" s="27"/>
       <c r="L5" s="26" t="s">
@@ -3735,13 +3762,15 @@
         <v>9.375</v>
       </c>
       <c r="S5" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T5" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="U5" s="27" t="s">
-        <v>85</v>
+      <c r="U5" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -3772,8 +3801,10 @@
       <c r="I6" s="29" t="s">
         <v>89</v>
       </c>
-      <c r="J6" s="29" t="s">
-        <v>73</v>
+      <c r="J6" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K6" s="18"/>
       <c r="L6" s="29" t="s">
@@ -3797,12 +3828,16 @@
         <v>5.625</v>
       </c>
       <c r="S6" s="29">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T6" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="U6" s="18"/>
+      <c r="U6" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="26" t="s">
@@ -3832,8 +3867,10 @@
       <c r="I7" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J7" s="26" t="s">
-        <v>73</v>
+      <c r="J7" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K7" s="27"/>
       <c r="L7" s="26" t="s">
@@ -3857,13 +3894,15 @@
         <v>5.625</v>
       </c>
       <c r="S7" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T7" s="27" t="s">
         <v>75</v>
       </c>
-      <c r="U7" s="27" t="s">
-        <v>94</v>
+      <c r="U7" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -3894,8 +3933,10 @@
       <c r="I8" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J8" s="26" t="s">
-        <v>73</v>
+      <c r="J8" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partially Complete</t>
+        </is>
       </c>
       <c r="K8" s="27"/>
       <c r="L8" s="26" t="s">
@@ -3919,11 +3960,13 @@
         <v>5</v>
       </c>
       <c r="S8" s="26">
-        <v>0.0</v>
+        <v>70</v>
       </c>
       <c r="T8" s="27"/>
-      <c r="U8" s="27" t="s">
-        <v>99</v>
+      <c r="U8" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metadata/runbook present and DocuSign configured. AWS Textract, Azure OCR, Virus Scan, and Adobe Sign secrets/endpoints still require subscriber setup.</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -3954,8 +3997,10 @@
       <c r="I9" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J9" s="26" t="s">
-        <v>73</v>
+      <c r="J9" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K9" s="27"/>
       <c r="L9" s="26" t="s">
@@ -3979,13 +4024,15 @@
         <v>15</v>
       </c>
       <c r="S9" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T9" s="27" t="s">
         <v>104</v>
       </c>
-      <c r="U9" s="27" t="s">
-        <v>105</v>
+      <c r="U9" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -4016,8 +4063,10 @@
       <c r="I10" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J10" s="26" t="s">
-        <v>73</v>
+      <c r="J10" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K10" s="27"/>
       <c r="L10" s="26" t="s">
@@ -4041,12 +4090,16 @@
         <v>9.375</v>
       </c>
       <c r="S10" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T10" s="27" t="s">
         <v>109</v>
       </c>
-      <c r="U10" s="27"/>
+      <c r="U10" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="26" t="s">
@@ -4076,8 +4129,10 @@
       <c r="I11" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J11" s="26" t="s">
-        <v>73</v>
+      <c r="J11" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K11" s="27"/>
       <c r="L11" s="26" t="s">
@@ -4101,13 +4156,15 @@
         <v>9.375</v>
       </c>
       <c r="S11" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T11" s="27" t="s">
         <v>113</v>
       </c>
-      <c r="U11" s="27" t="s">
-        <v>114</v>
+      <c r="U11" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -4138,8 +4195,10 @@
       <c r="I12" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J12" s="26" t="s">
-        <v>73</v>
+      <c r="J12" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K12" s="27"/>
       <c r="L12" s="26" t="s">
@@ -4163,12 +4222,16 @@
         <v>9.375</v>
       </c>
       <c r="S12" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T12" s="27" t="s">
         <v>100</v>
       </c>
-      <c r="U12" s="27"/>
+      <c r="U12" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="26" t="s">
@@ -4198,8 +4261,10 @@
       <c r="I13" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J13" s="26" t="s">
-        <v>73</v>
+      <c r="J13" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K13" s="27"/>
       <c r="L13" s="26" t="s">
@@ -4223,12 +4288,16 @@
         <v>9.375</v>
       </c>
       <c r="S13" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T13" s="27" t="s">
         <v>122</v>
       </c>
-      <c r="U13" s="27"/>
+      <c r="U13" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="26" t="s">
@@ -4258,8 +4327,10 @@
       <c r="I14" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J14" s="26" t="s">
-        <v>73</v>
+      <c r="J14" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K14" s="27"/>
       <c r="L14" s="26" t="s">
@@ -4283,13 +4354,15 @@
         <v>9.375</v>
       </c>
       <c r="S14" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T14" s="27" t="s">
         <v>126</v>
       </c>
-      <c r="U14" s="27" t="s">
-        <v>127</v>
+      <c r="U14" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -4320,8 +4393,10 @@
       <c r="I15" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J15" s="26" t="s">
-        <v>73</v>
+      <c r="J15" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K15" s="27"/>
       <c r="L15" s="26" t="s">
@@ -4345,13 +4420,15 @@
         <v>7.5</v>
       </c>
       <c r="S15" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T15" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="U15" s="27" t="s">
-        <v>131</v>
+      <c r="U15" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -4382,8 +4459,10 @@
       <c r="I16" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J16" s="26" t="s">
-        <v>73</v>
+      <c r="J16" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K16" s="27"/>
       <c r="L16" s="26" t="s">
@@ -4407,12 +4486,16 @@
         <v>15</v>
       </c>
       <c r="S16" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T16" s="27" t="s">
         <v>135</v>
       </c>
-      <c r="U16" s="27"/>
+      <c r="U16" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="26" t="s">
@@ -4442,8 +4525,10 @@
       <c r="I17" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J17" s="26" t="s">
-        <v>73</v>
+      <c r="J17" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K17" s="27"/>
       <c r="L17" s="26" t="s">
@@ -4467,13 +4552,15 @@
         <v>15</v>
       </c>
       <c r="S17" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T17" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="U17" s="27" t="s">
-        <v>140</v>
+      <c r="U17" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -4504,8 +4591,10 @@
       <c r="I18" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J18" s="26" t="s">
-        <v>73</v>
+      <c r="J18" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K18" s="27"/>
       <c r="L18" s="26" t="s">
@@ -4529,13 +4618,15 @@
         <v>15</v>
       </c>
       <c r="S18" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T18" s="27" t="s">
         <v>144</v>
       </c>
-      <c r="U18" s="27" t="s">
-        <v>145</v>
+      <c r="U18" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -4566,8 +4657,10 @@
       <c r="I19" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J19" s="26" t="s">
-        <v>73</v>
+      <c r="J19" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K19" s="27"/>
       <c r="L19" s="26" t="s">
@@ -4591,13 +4684,15 @@
         <v>9.375</v>
       </c>
       <c r="S19" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T19" s="27" t="s">
         <v>82</v>
       </c>
-      <c r="U19" s="27" t="s">
-        <v>149</v>
+      <c r="U19" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -4628,8 +4723,10 @@
       <c r="I20" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J20" s="26" t="s">
-        <v>73</v>
+      <c r="J20" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K20" s="27"/>
       <c r="L20" s="26" t="s">
@@ -4653,13 +4750,15 @@
         <v>15</v>
       </c>
       <c r="S20" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T20" s="27" t="s">
         <v>153</v>
       </c>
-      <c r="U20" s="27" t="s">
-        <v>154</v>
+      <c r="U20" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
@@ -4690,8 +4789,10 @@
       <c r="I21" s="29" t="s">
         <v>89</v>
       </c>
-      <c r="J21" s="29" t="s">
-        <v>73</v>
+      <c r="J21" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K21" s="18"/>
       <c r="L21" s="29" t="s">
@@ -4715,12 +4816,16 @@
         <v>9.375</v>
       </c>
       <c r="S21" s="29">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T21" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="U21" s="18"/>
+      <c r="U21" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="26" t="s">
@@ -4750,8 +4855,10 @@
       <c r="I22" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J22" s="26" t="s">
-        <v>73</v>
+      <c r="J22" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K22" s="27"/>
       <c r="L22" s="26" t="s">
@@ -4775,13 +4882,15 @@
         <v>12.5</v>
       </c>
       <c r="S22" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T22" s="27" t="s">
         <v>162</v>
       </c>
-      <c r="U22" s="27" t="s">
-        <v>163</v>
+      <c r="U22" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="23" ht="62.25" customHeight="1">
@@ -4812,8 +4921,10 @@
       <c r="I23" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J23" s="26" t="s">
-        <v>73</v>
+      <c r="J23" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K23" s="27"/>
       <c r="L23" s="26" t="s">
@@ -4837,13 +4948,15 @@
         <v>7.5</v>
       </c>
       <c r="S23" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T23" s="27" t="s">
         <v>110</v>
       </c>
-      <c r="U23" s="27" t="s">
-        <v>167</v>
+      <c r="U23" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
@@ -4874,8 +4987,10 @@
       <c r="I24" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J24" s="26" t="s">
-        <v>73</v>
+      <c r="J24" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K24" s="27"/>
       <c r="L24" s="26" t="s">
@@ -4899,13 +5014,15 @@
         <v>9.375</v>
       </c>
       <c r="S24" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T24" s="27" t="s">
         <v>171</v>
       </c>
-      <c r="U24" s="27" t="s">
-        <v>172</v>
+      <c r="U24" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
@@ -4936,8 +5053,10 @@
       <c r="I25" s="29" t="s">
         <v>89</v>
       </c>
-      <c r="J25" s="29" t="s">
-        <v>73</v>
+      <c r="J25" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K25" s="18"/>
       <c r="L25" s="29" t="s">
@@ -4961,12 +5080,16 @@
         <v>12.5</v>
       </c>
       <c r="S25" s="29">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T25" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="U25" s="18"/>
+      <c r="U25" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="26" t="s">
@@ -4996,8 +5119,10 @@
       <c r="I26" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J26" s="26" t="s">
-        <v>73</v>
+      <c r="J26" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K26" s="27"/>
       <c r="L26" s="26" t="s">
@@ -5021,12 +5146,16 @@
         <v>7.5</v>
       </c>
       <c r="S26" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T26" s="27" t="s">
         <v>179</v>
       </c>
-      <c r="U26" s="27"/>
+      <c r="U26" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="26" t="s">
@@ -5056,8 +5185,10 @@
       <c r="I27" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J27" s="26" t="s">
-        <v>73</v>
+      <c r="J27" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K27" s="27"/>
       <c r="L27" s="26" t="s">
@@ -5081,11 +5212,13 @@
         <v>5.625</v>
       </c>
       <c r="S27" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T27" s="27"/>
-      <c r="U27" s="27" t="s">
-        <v>183</v>
+      <c r="U27" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
@@ -5116,8 +5249,10 @@
       <c r="I28" s="29" t="s">
         <v>89</v>
       </c>
-      <c r="J28" s="29" t="s">
-        <v>73</v>
+      <c r="J28" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K28" s="18"/>
       <c r="L28" s="29" t="s">
@@ -5141,13 +5276,15 @@
         <v>15</v>
       </c>
       <c r="S28" s="29">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T28" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="U28" s="18" t="s">
-        <v>188</v>
+      <c r="U28" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
@@ -5178,8 +5315,10 @@
       <c r="I29" s="29" t="s">
         <v>89</v>
       </c>
-      <c r="J29" s="29" t="s">
-        <v>73</v>
+      <c r="J29" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K29" s="18"/>
       <c r="L29" s="29" t="s">
@@ -5203,12 +5342,16 @@
         <v>9.375</v>
       </c>
       <c r="S29" s="29">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T29" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="U29" s="18"/>
+      <c r="U29" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="26" t="s">
@@ -5238,8 +5381,10 @@
       <c r="I30" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J30" s="26" t="s">
-        <v>73</v>
+      <c r="J30" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K30" s="27"/>
       <c r="L30" s="26" t="s">
@@ -5263,13 +5408,15 @@
         <v>20</v>
       </c>
       <c r="S30" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T30" s="27" t="s">
         <v>196</v>
       </c>
-      <c r="U30" s="27" t="s">
-        <v>197</v>
+      <c r="U30" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
@@ -5300,8 +5447,10 @@
       <c r="I31" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J31" s="26" t="s">
-        <v>73</v>
+      <c r="J31" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K31" s="27"/>
       <c r="L31" s="26" t="s">
@@ -5325,13 +5474,15 @@
         <v>31.25</v>
       </c>
       <c r="S31" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T31" s="27" t="s">
         <v>192</v>
       </c>
-      <c r="U31" s="27" t="s">
-        <v>202</v>
+      <c r="U31" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
@@ -5362,8 +5513,10 @@
       <c r="I32" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="J32" s="30" t="s">
-        <v>73</v>
+      <c r="J32" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K32" s="20"/>
       <c r="L32" s="30" t="s">
@@ -5387,13 +5540,15 @@
         <v>5.625</v>
       </c>
       <c r="S32" s="30">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T32" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="U32" s="20" t="s">
-        <v>206</v>
+      <c r="U32" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
@@ -5424,8 +5579,10 @@
       <c r="I33" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="J33" s="30" t="s">
-        <v>73</v>
+      <c r="J33" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K33" s="20"/>
       <c r="L33" s="30" t="s">
@@ -5449,13 +5606,15 @@
         <v>15</v>
       </c>
       <c r="S33" s="30">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T33" s="20" t="s">
         <v>210</v>
       </c>
-      <c r="U33" s="20" t="s">
-        <v>211</v>
+      <c r="U33" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
@@ -5486,8 +5645,10 @@
       <c r="I34" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="J34" s="30" t="s">
-        <v>73</v>
+      <c r="J34" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K34" s="20"/>
       <c r="L34" s="30" t="s">
@@ -5511,12 +5672,16 @@
         <v>9.375</v>
       </c>
       <c r="S34" s="30">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T34" s="20" t="s">
         <v>207</v>
       </c>
-      <c r="U34" s="20"/>
+      <c r="U34" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="30" t="s">
@@ -5546,8 +5711,10 @@
       <c r="I35" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="J35" s="30" t="s">
-        <v>73</v>
+      <c r="J35" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K35" s="20"/>
       <c r="L35" s="30" t="s">
@@ -5571,13 +5738,15 @@
         <v>5.625</v>
       </c>
       <c r="S35" s="30">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T35" s="20" t="s">
         <v>207</v>
       </c>
-      <c r="U35" s="20" t="s">
-        <v>218</v>
+      <c r="U35" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
@@ -5608,8 +5777,10 @@
       <c r="I36" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="J36" s="30" t="s">
-        <v>73</v>
+      <c r="J36" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K36" s="20"/>
       <c r="L36" s="30" t="s">
@@ -5633,12 +5804,16 @@
         <v>15</v>
       </c>
       <c r="S36" s="30">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T36" s="20" t="s">
         <v>207</v>
       </c>
-      <c r="U36" s="20"/>
+      <c r="U36" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="30" t="s">
@@ -5668,8 +5843,10 @@
       <c r="I37" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="J37" s="30" t="s">
-        <v>73</v>
+      <c r="J37" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K37" s="20"/>
       <c r="L37" s="30" t="s">
@@ -5693,12 +5870,16 @@
         <v>7.5</v>
       </c>
       <c r="S37" s="30">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T37" s="20" t="s">
         <v>225</v>
       </c>
-      <c r="U37" s="20"/>
+      <c r="U37" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="30" t="s">
@@ -5728,8 +5909,10 @@
       <c r="I38" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="J38" s="30" t="s">
-        <v>73</v>
+      <c r="J38" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K38" s="20"/>
       <c r="L38" s="30" t="s">
@@ -5753,13 +5936,15 @@
         <v>12.5</v>
       </c>
       <c r="S38" s="30">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T38" s="20" t="s">
         <v>230</v>
       </c>
-      <c r="U38" s="20" t="s">
-        <v>231</v>
+      <c r="U38" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
@@ -5790,8 +5975,10 @@
       <c r="I39" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="J39" s="30" t="s">
-        <v>73</v>
+      <c r="J39" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K39" s="20"/>
       <c r="L39" s="30" t="s">
@@ -5815,13 +6002,15 @@
         <v>12.5</v>
       </c>
       <c r="S39" s="30">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T39" s="20" t="s">
         <v>226</v>
       </c>
-      <c r="U39" s="20" t="s">
-        <v>235</v>
+      <c r="U39" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
@@ -5852,8 +6041,10 @@
       <c r="I40" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="J40" s="30" t="s">
-        <v>73</v>
+      <c r="J40" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K40" s="20"/>
       <c r="L40" s="30" t="s">
@@ -5877,13 +6068,15 @@
         <v>12.5</v>
       </c>
       <c r="S40" s="30">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T40" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="U40" s="20" t="s">
-        <v>240</v>
+      <c r="U40" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
@@ -5914,8 +6107,10 @@
       <c r="I41" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="J41" s="30" t="s">
-        <v>73</v>
+      <c r="J41" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K41" s="20"/>
       <c r="L41" s="30" t="s">
@@ -5939,13 +6134,15 @@
         <v>15</v>
       </c>
       <c r="S41" s="30">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T41" s="20" t="s">
         <v>244</v>
       </c>
-      <c r="U41" s="20" t="s">
-        <v>245</v>
+      <c r="U41" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
@@ -5976,8 +6173,10 @@
       <c r="I42" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="J42" s="30" t="s">
-        <v>73</v>
+      <c r="J42" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K42" s="20"/>
       <c r="L42" s="30" t="s">
@@ -6001,13 +6200,15 @@
         <v>20</v>
       </c>
       <c r="S42" s="30">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T42" s="20" t="s">
         <v>249</v>
       </c>
-      <c r="U42" s="20" t="s">
-        <v>250</v>
+      <c r="U42" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
@@ -6038,8 +6239,10 @@
       <c r="I43" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="J43" s="30" t="s">
-        <v>73</v>
+      <c r="J43" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K43" s="20"/>
       <c r="L43" s="30" t="s">
@@ -6063,12 +6266,16 @@
         <v>12.5</v>
       </c>
       <c r="S43" s="30">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T43" s="20" t="s">
         <v>246</v>
       </c>
-      <c r="U43" s="20"/>
+      <c r="U43" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="30" t="s">
@@ -6098,8 +6305,10 @@
       <c r="I44" s="30" t="s">
         <v>257</v>
       </c>
-      <c r="J44" s="30" t="s">
-        <v>73</v>
+      <c r="J44" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paused</t>
+        </is>
       </c>
       <c r="K44" s="20"/>
       <c r="L44" s="30" t="s">
@@ -6123,13 +6332,15 @@
         <v>20</v>
       </c>
       <c r="S44" s="30">
-        <v>0.0</v>
+        <v>80</v>
       </c>
       <c r="T44" s="20" t="s">
         <v>249</v>
       </c>
-      <c r="U44" s="20" t="s">
-        <v>258</v>
+      <c r="U44" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adobe Sign service code and tests are complete. Live Adobe provider setup is paused because DocuSign is the selected demo provider.</t>
+        </is>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
@@ -6160,8 +6371,10 @@
       <c r="I45" s="30" t="s">
         <v>257</v>
       </c>
-      <c r="J45" s="30" t="s">
-        <v>73</v>
+      <c r="J45" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paused</t>
+        </is>
       </c>
       <c r="K45" s="20"/>
       <c r="L45" s="30" t="s">
@@ -6185,12 +6398,16 @@
         <v>7.5</v>
       </c>
       <c r="S45" s="30">
-        <v>0.0</v>
+        <v>80</v>
       </c>
       <c r="T45" s="20" t="s">
         <v>254</v>
       </c>
-      <c r="U45" s="20"/>
+      <c r="U45" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adobe Sign webhook code and tests are complete. Live Adobe webhook/provider setup is paused unless Adobe Sign is selected.</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="30" t="s">
@@ -6220,8 +6437,10 @@
       <c r="I46" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="J46" s="30" t="s">
-        <v>73</v>
+      <c r="J46" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K46" s="20"/>
       <c r="L46" s="30" t="s">
@@ -6245,13 +6464,15 @@
         <v>9.375</v>
       </c>
       <c r="S46" s="30">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T46" s="20" t="s">
         <v>265</v>
       </c>
-      <c r="U46" s="20" t="s">
-        <v>266</v>
+      <c r="U46" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
@@ -6282,8 +6503,10 @@
       <c r="I47" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="J47" s="30" t="s">
-        <v>73</v>
+      <c r="J47" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K47" s="20"/>
       <c r="L47" s="30" t="s">
@@ -6307,13 +6530,15 @@
         <v>6.25</v>
       </c>
       <c r="S47" s="30">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T47" s="20" t="s">
         <v>244</v>
       </c>
-      <c r="U47" s="20" t="s">
-        <v>270</v>
+      <c r="U47" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
@@ -6344,8 +6569,10 @@
       <c r="I48" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="J48" s="30" t="s">
-        <v>73</v>
+      <c r="J48" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K48" s="20"/>
       <c r="L48" s="30" t="s">
@@ -6369,13 +6596,15 @@
         <v>12.5</v>
       </c>
       <c r="S48" s="30">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T48" s="20" t="s">
         <v>109</v>
       </c>
-      <c r="U48" s="20" t="s">
-        <v>275</v>
+      <c r="U48" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
@@ -6406,8 +6635,10 @@
       <c r="I49" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="J49" s="30" t="s">
-        <v>73</v>
+      <c r="J49" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K49" s="20"/>
       <c r="L49" s="30" t="s">
@@ -6431,13 +6662,15 @@
         <v>20</v>
       </c>
       <c r="S49" s="30">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T49" s="20" t="s">
         <v>279</v>
       </c>
-      <c r="U49" s="20" t="s">
-        <v>280</v>
+      <c r="U49" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
@@ -6468,8 +6701,10 @@
       <c r="I50" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="J50" s="30" t="s">
-        <v>73</v>
+      <c r="J50" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K50" s="20"/>
       <c r="L50" s="30" t="s">
@@ -6493,12 +6728,16 @@
         <v>25</v>
       </c>
       <c r="S50" s="30">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T50" s="20" t="s">
         <v>276</v>
       </c>
-      <c r="U50" s="20"/>
+      <c r="U50" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="31" t="s">
@@ -6528,8 +6767,10 @@
       <c r="I51" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="J51" s="31" t="s">
-        <v>73</v>
+      <c r="J51" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K51" s="22"/>
       <c r="L51" s="31" t="s">
@@ -6553,13 +6794,15 @@
         <v>12.5</v>
       </c>
       <c r="S51" s="31">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T51" s="22" t="s">
         <v>287</v>
       </c>
-      <c r="U51" s="22" t="s">
-        <v>288</v>
+      <c r="U51" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
@@ -6590,8 +6833,10 @@
       <c r="I52" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="J52" s="31" t="s">
-        <v>73</v>
+      <c r="J52" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Needs Review</t>
+        </is>
       </c>
       <c r="K52" s="22"/>
       <c r="L52" s="31" t="s">
@@ -6615,12 +6860,16 @@
         <v>12.5</v>
       </c>
       <c r="S52" s="31">
-        <v>0.0</v>
+        <v>50</v>
       </c>
       <c r="T52" s="22" t="s">
         <v>292</v>
       </c>
-      <c r="U52" s="22"/>
+      <c r="U52" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tracker asks for kt_verify_document. Implemented MCP tool is kt_upload_document instead; verify tool scope needs product decision or rename.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="31" t="s">
@@ -6650,8 +6899,10 @@
       <c r="I53" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="J53" s="31" t="s">
-        <v>73</v>
+      <c r="J53" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K53" s="22"/>
       <c r="L53" s="31" t="s">
@@ -6675,12 +6926,16 @@
         <v>7.5</v>
       </c>
       <c r="S53" s="31">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T53" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="U53" s="22"/>
+      <c r="U53" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="31" t="s">
@@ -6710,8 +6965,10 @@
       <c r="I54" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="J54" s="31" t="s">
-        <v>73</v>
+      <c r="J54" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K54" s="22"/>
       <c r="L54" s="31" t="s">
@@ -6735,12 +6992,16 @@
         <v>7.5</v>
       </c>
       <c r="S54" s="31">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T54" s="22" t="s">
         <v>141</v>
       </c>
-      <c r="U54" s="22"/>
+      <c r="U54" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="31" t="s">
@@ -6770,8 +7031,10 @@
       <c r="I55" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="J55" s="31" t="s">
-        <v>73</v>
+      <c r="J55" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partially Complete</t>
+        </is>
       </c>
       <c r="K55" s="22"/>
       <c r="L55" s="31" t="s">
@@ -6795,12 +7058,16 @@
         <v>15.625</v>
       </c>
       <c r="S55" s="31">
-        <v>0.0</v>
+        <v>80</v>
       </c>
       <c r="T55" s="22" t="s">
         <v>302</v>
       </c>
-      <c r="U55" s="22"/>
+      <c r="U55" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MCP request/get/dispatch/upload flows implemented. Sprint 7 UAT is pending tracker alignment for kt_verify_document vs kt_upload_document.</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="32" t="s">
@@ -6830,8 +7097,10 @@
       <c r="I56" s="32" t="s">
         <v>89</v>
       </c>
-      <c r="J56" s="32" t="s">
-        <v>73</v>
+      <c r="J56" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K56" s="24"/>
       <c r="L56" s="32" t="s">
@@ -6855,12 +7124,16 @@
         <v>7.5</v>
       </c>
       <c r="S56" s="32">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T56" s="24" t="s">
         <v>153</v>
       </c>
-      <c r="U56" s="24"/>
+      <c r="U56" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="32" t="s">
@@ -6890,8 +7163,10 @@
       <c r="I57" s="32" t="s">
         <v>89</v>
       </c>
-      <c r="J57" s="32" t="s">
-        <v>73</v>
+      <c r="J57" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K57" s="24"/>
       <c r="L57" s="32" t="s">
@@ -6915,13 +7190,15 @@
         <v>12.5</v>
       </c>
       <c r="S57" s="32">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T57" s="24" t="s">
         <v>303</v>
       </c>
-      <c r="U57" s="24" t="s">
-        <v>309</v>
+      <c r="U57" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
@@ -6952,8 +7229,10 @@
       <c r="I58" s="32" t="s">
         <v>89</v>
       </c>
-      <c r="J58" s="32" t="s">
-        <v>73</v>
+      <c r="J58" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K58" s="24"/>
       <c r="L58" s="32" t="s">
@@ -6977,13 +7256,15 @@
         <v>12.5</v>
       </c>
       <c r="S58" s="32">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T58" s="24" t="s">
         <v>153</v>
       </c>
-      <c r="U58" s="24" t="s">
-        <v>313</v>
+      <c r="U58" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
@@ -7014,8 +7295,10 @@
       <c r="I59" s="32" t="s">
         <v>257</v>
       </c>
-      <c r="J59" s="32" t="s">
-        <v>73</v>
+      <c r="J59" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Deferred</t>
+        </is>
       </c>
       <c r="K59" s="24"/>
       <c r="L59" s="32" t="s">
@@ -7039,13 +7322,15 @@
         <v>12.5</v>
       </c>
       <c r="S59" s="32">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="T59" s="24" t="s">
         <v>317</v>
       </c>
-      <c r="U59" s="24" t="s">
-        <v>318</v>
+      <c r="U59" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Optional AgentExchange DocuSign connector upgrade deferred; package/connector access and tenant setup are not available. Custom DocuSign Named Credential integration remains active.</t>
+        </is>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
@@ -7076,8 +7361,10 @@
       <c r="I60" s="32" t="s">
         <v>89</v>
       </c>
-      <c r="J60" s="32" t="s">
-        <v>73</v>
+      <c r="J60" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K60" s="24"/>
       <c r="L60" s="32" t="s">
@@ -7101,12 +7388,16 @@
         <v>15.625</v>
       </c>
       <c r="S60" s="32">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T60" s="24" t="s">
         <v>322</v>
       </c>
-      <c r="U60" s="24"/>
+      <c r="U60" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="26" t="s">
@@ -7136,8 +7427,10 @@
       <c r="I61" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="J61" s="26" t="s">
-        <v>73</v>
+      <c r="J61" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed</t>
+        </is>
       </c>
       <c r="K61" s="27"/>
       <c r="L61" s="26" t="s">
@@ -7161,13 +7454,15 @@
         <v>31.25</v>
       </c>
       <c r="S61" s="26">
-        <v>0.0</v>
+        <v>100</v>
       </c>
       <c r="T61" s="27" t="s">
         <v>326</v>
       </c>
-      <c r="U61" s="27" t="s">
-        <v>327</v>
+      <c r="U61" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Completed in implementation; see docs/implementation/KT_B4_Development_Status.md and related implementation/UAT docs.</t>
+        </is>
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1"/>
@@ -8118,7 +8413,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <pageSetUpPr/>
@@ -10564,7 +10859,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <pageSetUpPr/>

</xml_diff>